<commit_message>
Added miscrosoft and google income statements
</commit_message>
<xml_diff>
--- a/Apple 2009-2024.xlsx
+++ b/Apple 2009-2024.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HAZEL\Desktop\GenData_Capstone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{769407A4-3023-4EE9-8E0F-743345321E08}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{2B85EE23-DA0D-40E7-9BA4-BC3C8280D817}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810"/>
   </bookViews>
   <sheets>
     <sheet name="Apple 2009-2024" sheetId="1" r:id="rId1"/>
+    <sheet name="microsoft income statement" sheetId="3" r:id="rId2"/>
+    <sheet name="Google-Alphabet income " sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="464">
   <si>
     <t>year</t>
   </si>
@@ -539,13 +541,886 @@
   </si>
   <si>
     <t>$15,861</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>$281,724</t>
+  </si>
+  <si>
+    <t>$245,122</t>
+  </si>
+  <si>
+    <t>$211,915</t>
+  </si>
+  <si>
+    <t>$198,270</t>
+  </si>
+  <si>
+    <t>$168,088</t>
+  </si>
+  <si>
+    <t>$143,015</t>
+  </si>
+  <si>
+    <t>$125,843</t>
+  </si>
+  <si>
+    <t>$110,360</t>
+  </si>
+  <si>
+    <t>$96,571</t>
+  </si>
+  <si>
+    <t>$91,154</t>
+  </si>
+  <si>
+    <t>$93,580</t>
+  </si>
+  <si>
+    <t>$86,833</t>
+  </si>
+  <si>
+    <t>$77,849</t>
+  </si>
+  <si>
+    <t>$73,723</t>
+  </si>
+  <si>
+    <t>$69,940</t>
+  </si>
+  <si>
+    <t>EBITDA (Millions of US $)</t>
+  </si>
+  <si>
+    <t>$162,681</t>
+  </si>
+  <si>
+    <t>$131,720</t>
+  </si>
+  <si>
+    <t>$102,384</t>
+  </si>
+  <si>
+    <t>$97,843</t>
+  </si>
+  <si>
+    <t>$81,602</t>
+  </si>
+  <si>
+    <t>$65,755</t>
+  </si>
+  <si>
+    <t>$54,641</t>
+  </si>
+  <si>
+    <t>$45,319</t>
+  </si>
+  <si>
+    <t>$37,803</t>
+  </si>
+  <si>
+    <t>$33,330</t>
+  </si>
+  <si>
+    <t>$31,616</t>
+  </si>
+  <si>
+    <t>$32,971</t>
+  </si>
+  <si>
+    <t>$30,519</t>
+  </si>
+  <si>
+    <t>$30,923</t>
+  </si>
+  <si>
+    <t>$29,927</t>
+  </si>
+  <si>
+    <t>Gross Profit (Millions of US $)</t>
+  </si>
+  <si>
+    <t>$193,893</t>
+  </si>
+  <si>
+    <t>$171,008</t>
+  </si>
+  <si>
+    <t>$146,052</t>
+  </si>
+  <si>
+    <t>$135,620</t>
+  </si>
+  <si>
+    <t>$115,856</t>
+  </si>
+  <si>
+    <t>$96,937</t>
+  </si>
+  <si>
+    <t>$82,933</t>
+  </si>
+  <si>
+    <t>$72,007</t>
+  </si>
+  <si>
+    <t>$62,310</t>
+  </si>
+  <si>
+    <t>$58,374</t>
+  </si>
+  <si>
+    <t>$60,542</t>
+  </si>
+  <si>
+    <t>$59,755</t>
+  </si>
+  <si>
+    <t>$57,464</t>
+  </si>
+  <si>
+    <t>$56,193</t>
+  </si>
+  <si>
+    <t>$54,366</t>
+  </si>
+  <si>
+    <t>Operating Income (Millions of US $)</t>
+  </si>
+  <si>
+    <t>$128,528</t>
+  </si>
+  <si>
+    <t>$109,433</t>
+  </si>
+  <si>
+    <t>$88,523</t>
+  </si>
+  <si>
+    <t>$83,383</t>
+  </si>
+  <si>
+    <t>$69,916</t>
+  </si>
+  <si>
+    <t>$52,959</t>
+  </si>
+  <si>
+    <t>$42,959</t>
+  </si>
+  <si>
+    <t>$35,058</t>
+  </si>
+  <si>
+    <t>$29,025</t>
+  </si>
+  <si>
+    <t>$26,078</t>
+  </si>
+  <si>
+    <t>$18,161</t>
+  </si>
+  <si>
+    <t>$27,759</t>
+  </si>
+  <si>
+    <t>$26,764</t>
+  </si>
+  <si>
+    <t>$21,763</t>
+  </si>
+  <si>
+    <t>$27,161</t>
+  </si>
+  <si>
+    <t>Net Income (Millions of US $)</t>
+  </si>
+  <si>
+    <t>$101,832</t>
+  </si>
+  <si>
+    <t>$88,136</t>
+  </si>
+  <si>
+    <t>$72,361</t>
+  </si>
+  <si>
+    <t>$72,738</t>
+  </si>
+  <si>
+    <t>$61,271</t>
+  </si>
+  <si>
+    <t>$44,281</t>
+  </si>
+  <si>
+    <t>$39,240</t>
+  </si>
+  <si>
+    <t>$16,571</t>
+  </si>
+  <si>
+    <t>$25,489</t>
+  </si>
+  <si>
+    <t>$20,539</t>
+  </si>
+  <si>
+    <t>$12,193</t>
+  </si>
+  <si>
+    <t>$22,074</t>
+  </si>
+  <si>
+    <t>$21,863</t>
+  </si>
+  <si>
+    <t>$16,978</t>
+  </si>
+  <si>
+    <t>$23,150</t>
+  </si>
+  <si>
+    <t>$13.64</t>
+  </si>
+  <si>
+    <t>$11.80</t>
+  </si>
+  <si>
+    <t>$9.68</t>
+  </si>
+  <si>
+    <t>$9.65</t>
+  </si>
+  <si>
+    <t>$8.05</t>
+  </si>
+  <si>
+    <t>$5.76</t>
+  </si>
+  <si>
+    <t>$5.06</t>
+  </si>
+  <si>
+    <t>$2.13</t>
+  </si>
+  <si>
+    <t>$3.25</t>
+  </si>
+  <si>
+    <t>$2.56</t>
+  </si>
+  <si>
+    <t>$1.48</t>
+  </si>
+  <si>
+    <t>$2.63</t>
+  </si>
+  <si>
+    <t>$2.58</t>
+  </si>
+  <si>
+    <t>$2.00</t>
+  </si>
+  <si>
+    <t>$2.69</t>
+  </si>
+  <si>
+    <t>Shares Outstanding (Millions)</t>
+  </si>
+  <si>
+    <t>Total Assets (Millions)</t>
+  </si>
+  <si>
+    <t>$619,003</t>
+  </si>
+  <si>
+    <t>$512,163</t>
+  </si>
+  <si>
+    <t>$411,976</t>
+  </si>
+  <si>
+    <t>$364,840</t>
+  </si>
+  <si>
+    <t>$333,779</t>
+  </si>
+  <si>
+    <t>$301,311</t>
+  </si>
+  <si>
+    <t>$286,556</t>
+  </si>
+  <si>
+    <t>$258,848</t>
+  </si>
+  <si>
+    <t>$250,312</t>
+  </si>
+  <si>
+    <t>$193,468</t>
+  </si>
+  <si>
+    <t>$174,472</t>
+  </si>
+  <si>
+    <t>$172,384</t>
+  </si>
+  <si>
+    <t>$142,431</t>
+  </si>
+  <si>
+    <t>$121,271</t>
+  </si>
+  <si>
+    <t>$108,704</t>
+  </si>
+  <si>
+    <t>Cash on Hand (Millions)</t>
+  </si>
+  <si>
+    <t>$94,565</t>
+  </si>
+  <si>
+    <t>$75,543</t>
+  </si>
+  <si>
+    <t>$111,262</t>
+  </si>
+  <si>
+    <t>$104,757</t>
+  </si>
+  <si>
+    <t>$130,334</t>
+  </si>
+  <si>
+    <t>$136,527</t>
+  </si>
+  <si>
+    <t>$133,819</t>
+  </si>
+  <si>
+    <t>$133,768</t>
+  </si>
+  <si>
+    <t>$132,981</t>
+  </si>
+  <si>
+    <t>$113,240</t>
+  </si>
+  <si>
+    <t>$96,526</t>
+  </si>
+  <si>
+    <t>$85,709</t>
+  </si>
+  <si>
+    <t>$77,022</t>
+  </si>
+  <si>
+    <t>$63,040</t>
+  </si>
+  <si>
+    <t>$52,772</t>
+  </si>
+  <si>
+    <t>Long Term Debt (Millions of US $)</t>
+  </si>
+  <si>
+    <t>Total Liabilities (Millions of US $)</t>
+  </si>
+  <si>
+    <t>PE Ratio</t>
+  </si>
+  <si>
+    <t>Employee Count</t>
+  </si>
+  <si>
+    <t>$402,836</t>
+  </si>
+  <si>
+    <t>$350,018</t>
+  </si>
+  <si>
+    <t>$307,394</t>
+  </si>
+  <si>
+    <t>$282,836</t>
+  </si>
+  <si>
+    <t>$257,637</t>
+  </si>
+  <si>
+    <t>$182,527</t>
+  </si>
+  <si>
+    <t>$161,857</t>
+  </si>
+  <si>
+    <t>$136,819</t>
+  </si>
+  <si>
+    <t>$110,855</t>
+  </si>
+  <si>
+    <t>$90,272</t>
+  </si>
+  <si>
+    <t>$74,989</t>
+  </si>
+  <si>
+    <t>$66,001</t>
+  </si>
+  <si>
+    <t>$55,519</t>
+  </si>
+  <si>
+    <t>$46,039</t>
+  </si>
+  <si>
+    <t>$37,905</t>
+  </si>
+  <si>
+    <t>EBITDA</t>
+  </si>
+  <si>
+    <t>$150,175</t>
+  </si>
+  <si>
+    <t>$127,701</t>
+  </si>
+  <si>
+    <t>$96,239</t>
+  </si>
+  <si>
+    <t>$88,317</t>
+  </si>
+  <si>
+    <t>$88,987</t>
+  </si>
+  <si>
+    <t>$54,921</t>
+  </si>
+  <si>
+    <t>$46,012</t>
+  </si>
+  <si>
+    <t>$36,559</t>
+  </si>
+  <si>
+    <t>$33,093</t>
+  </si>
+  <si>
+    <t>$29,860</t>
+  </si>
+  <si>
+    <t>$24,423</t>
+  </si>
+  <si>
+    <t>$21,475</t>
+  </si>
+  <si>
+    <t>$19,342</t>
+  </si>
+  <si>
+    <t>$16,796</t>
+  </si>
+  <si>
+    <t>$13,593</t>
+  </si>
+  <si>
+    <t>Gross Profit</t>
+  </si>
+  <si>
+    <t>$240,301</t>
+  </si>
+  <si>
+    <t>$203,712</t>
+  </si>
+  <si>
+    <t>$174,062</t>
+  </si>
+  <si>
+    <t>$156,633</t>
+  </si>
+  <si>
+    <t>$146,698</t>
+  </si>
+  <si>
+    <t>$97,795</t>
+  </si>
+  <si>
+    <t>$89,961</t>
+  </si>
+  <si>
+    <t>$77,270</t>
+  </si>
+  <si>
+    <t>$65,272</t>
+  </si>
+  <si>
+    <t>$55,134</t>
+  </si>
+  <si>
+    <t>$46,825</t>
+  </si>
+  <si>
+    <t>$40,310</t>
+  </si>
+  <si>
+    <t>$33,526</t>
+  </si>
+  <si>
+    <t>$28,863</t>
+  </si>
+  <si>
+    <t>$24,717</t>
+  </si>
+  <si>
+    <t>Operating Income</t>
+  </si>
+  <si>
+    <t>$129,039</t>
+  </si>
+  <si>
+    <t>$112,390</t>
+  </si>
+  <si>
+    <t>$84,293</t>
+  </si>
+  <si>
+    <t>$74,842</t>
+  </si>
+  <si>
+    <t>$78,714</t>
+  </si>
+  <si>
+    <t>$41,224</t>
+  </si>
+  <si>
+    <t>$34,231</t>
+  </si>
+  <si>
+    <t>$27,524</t>
+  </si>
+  <si>
+    <t>$26,178</t>
+  </si>
+  <si>
+    <t>$23,716</t>
+  </si>
+  <si>
+    <t>$19,360</t>
+  </si>
+  <si>
+    <t>$16,496</t>
+  </si>
+  <si>
+    <t>$15,403</t>
+  </si>
+  <si>
+    <t>$13,834</t>
+  </si>
+  <si>
+    <t>$11,742</t>
+  </si>
+  <si>
+    <t>Net Income</t>
+  </si>
+  <si>
+    <t>$132,170</t>
+  </si>
+  <si>
+    <t>$100,118</t>
+  </si>
+  <si>
+    <t>$73,795</t>
+  </si>
+  <si>
+    <t>$59,972</t>
+  </si>
+  <si>
+    <t>$76,033</t>
+  </si>
+  <si>
+    <t>$40,269</t>
+  </si>
+  <si>
+    <t>$34,343</t>
+  </si>
+  <si>
+    <t>$30,736</t>
+  </si>
+  <si>
+    <t>$12,662</t>
+  </si>
+  <si>
+    <t>$19,478</t>
+  </si>
+  <si>
+    <t>$15,826</t>
+  </si>
+  <si>
+    <t>$14,136</t>
+  </si>
+  <si>
+    <t>$12,733</t>
+  </si>
+  <si>
+    <t>$10,737</t>
+  </si>
+  <si>
+    <t>$9,737</t>
+  </si>
+  <si>
+    <t>$10.81</t>
+  </si>
+  <si>
+    <t>$8.04</t>
+  </si>
+  <si>
+    <t>$5.80</t>
+  </si>
+  <si>
+    <t>$4.56</t>
+  </si>
+  <si>
+    <t>$2.93</t>
+  </si>
+  <si>
+    <t>$2.46</t>
+  </si>
+  <si>
+    <t>$2.19</t>
+  </si>
+  <si>
+    <t>$0.90</t>
+  </si>
+  <si>
+    <t>$1.39</t>
+  </si>
+  <si>
+    <t>$1.14</t>
+  </si>
+  <si>
+    <t>$1.03</t>
+  </si>
+  <si>
+    <t>$0.94</t>
+  </si>
+  <si>
+    <t>$0.81</t>
+  </si>
+  <si>
+    <t>$0.74</t>
+  </si>
+  <si>
+    <t>Year Close</t>
+  </si>
+  <si>
+    <t>Total Assets</t>
+  </si>
+  <si>
+    <t>$595,281</t>
+  </si>
+  <si>
+    <t>$450,256</t>
+  </si>
+  <si>
+    <t>$402,392</t>
+  </si>
+  <si>
+    <t>$365,264</t>
+  </si>
+  <si>
+    <t>$359,268</t>
+  </si>
+  <si>
+    <t>$319,616</t>
+  </si>
+  <si>
+    <t>$275,909</t>
+  </si>
+  <si>
+    <t>$232,792</t>
+  </si>
+  <si>
+    <t>$197,295</t>
+  </si>
+  <si>
+    <t>$167,497</t>
+  </si>
+  <si>
+    <t>$147,461</t>
+  </si>
+  <si>
+    <t>$129,187</t>
+  </si>
+  <si>
+    <t>$110,920</t>
+  </si>
+  <si>
+    <t>$93,798</t>
+  </si>
+  <si>
+    <t>$72,574</t>
+  </si>
+  <si>
+    <t>Cash on Hand</t>
+  </si>
+  <si>
+    <t>$126,843</t>
+  </si>
+  <si>
+    <t>$95,657</t>
+  </si>
+  <si>
+    <t>$110,916</t>
+  </si>
+  <si>
+    <t>$113,762</t>
+  </si>
+  <si>
+    <t>$139,649</t>
+  </si>
+  <si>
+    <t>$136,694</t>
+  </si>
+  <si>
+    <t>$119,675</t>
+  </si>
+  <si>
+    <t>$109,140</t>
+  </si>
+  <si>
+    <t>$101,871</t>
+  </si>
+  <si>
+    <t>$86,333</t>
+  </si>
+  <si>
+    <t>$73,066</t>
+  </si>
+  <si>
+    <t>$64,395</t>
+  </si>
+  <si>
+    <t>$58,717</t>
+  </si>
+  <si>
+    <t>$48,088</t>
+  </si>
+  <si>
+    <t>$44,626</t>
+  </si>
+  <si>
+    <t>Long Term Debt</t>
+  </si>
+  <si>
+    <t>$46,547</t>
+  </si>
+  <si>
+    <t>$10,883</t>
+  </si>
+  <si>
+    <t>$11,870</t>
+  </si>
+  <si>
+    <t>$14,701</t>
+  </si>
+  <si>
+    <t>$14,817</t>
+  </si>
+  <si>
+    <t>$13,932</t>
+  </si>
+  <si>
+    <t>$4,554</t>
+  </si>
+  <si>
+    <t>$4,012</t>
+  </si>
+  <si>
+    <t>$3,969</t>
+  </si>
+  <si>
+    <t>$3,935</t>
+  </si>
+  <si>
+    <t>$1,995</t>
+  </si>
+  <si>
+    <t>$3,228</t>
+  </si>
+  <si>
+    <t>$2,236</t>
+  </si>
+  <si>
+    <t>$2,988</t>
+  </si>
+  <si>
+    <t>$2,986</t>
+  </si>
+  <si>
+    <t>Total Liabilities</t>
+  </si>
+  <si>
+    <t>$180,016</t>
+  </si>
+  <si>
+    <t>$125,172</t>
+  </si>
+  <si>
+    <t>$119,013</t>
+  </si>
+  <si>
+    <t>$109,120</t>
+  </si>
+  <si>
+    <t>$107,633</t>
+  </si>
+  <si>
+    <t>$97,072</t>
+  </si>
+  <si>
+    <t>$74,467</t>
+  </si>
+  <si>
+    <t>$55,164</t>
+  </si>
+  <si>
+    <t>$44,793</t>
+  </si>
+  <si>
+    <t>$28,461</t>
+  </si>
+  <si>
+    <t>$27,130</t>
+  </si>
+  <si>
+    <t>$25,327</t>
+  </si>
+  <si>
+    <t>$23,611</t>
+  </si>
+  <si>
+    <t>$22,083</t>
+  </si>
+  <si>
+    <t>$14,429</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -680,8 +1555,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -861,8 +1750,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -977,6 +1872,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1022,10 +1932,45 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1383,9 +2328,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.90625" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1435,7 +2398,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2">
+      <c r="A2" s="15">
         <v>2024</v>
       </c>
       <c r="B2" t="s">
@@ -1485,7 +2448,7 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A3">
+      <c r="A3" s="15">
         <v>2023</v>
       </c>
       <c r="B3" t="s">
@@ -1535,7 +2498,7 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4">
+      <c r="A4" s="15">
         <v>2022</v>
       </c>
       <c r="B4" t="s">
@@ -1585,7 +2548,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5">
+      <c r="A5" s="15">
         <v>2021</v>
       </c>
       <c r="B5" t="s">
@@ -1635,7 +2598,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A6">
+      <c r="A6" s="15">
         <v>2020</v>
       </c>
       <c r="B6" t="s">
@@ -1685,7 +2648,7 @@
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A7">
+      <c r="A7" s="15">
         <v>2019</v>
       </c>
       <c r="B7" t="s">
@@ -1735,7 +2698,7 @@
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A8">
+      <c r="A8" s="15">
         <v>2018</v>
       </c>
       <c r="B8" t="s">
@@ -1785,7 +2748,7 @@
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A9">
+      <c r="A9" s="15">
         <v>2017</v>
       </c>
       <c r="B9" t="s">
@@ -1835,7 +2798,7 @@
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A10">
+      <c r="A10" s="15">
         <v>2016</v>
       </c>
       <c r="B10" t="s">
@@ -1885,7 +2848,7 @@
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A11">
+      <c r="A11" s="15">
         <v>2015</v>
       </c>
       <c r="B11" t="s">
@@ -1935,7 +2898,7 @@
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A12">
+      <c r="A12" s="15">
         <v>2014</v>
       </c>
       <c r="B12" t="s">
@@ -1985,7 +2948,7 @@
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A13">
+      <c r="A13" s="15">
         <v>2013</v>
       </c>
       <c r="B13" t="s">
@@ -2035,7 +2998,7 @@
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A14">
+      <c r="A14" s="15">
         <v>2012</v>
       </c>
       <c r="B14" t="s">
@@ -2085,7 +3048,7 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A15">
+      <c r="A15" s="15">
         <v>2011</v>
       </c>
       <c r="B15" t="s">
@@ -2135,7 +3098,7 @@
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A16">
+      <c r="A16" s="15">
         <v>2010</v>
       </c>
       <c r="B16" t="s">
@@ -2185,7 +3148,7 @@
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A17">
+      <c r="A17" s="15">
         <v>2009</v>
       </c>
       <c r="B17" t="s">
@@ -2232,6 +3195,1589 @@
       </c>
       <c r="P17" s="1">
         <v>36800</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:P16"/>
+  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.90625" style="7" customWidth="1"/>
+    <col min="2" max="7" width="8.7265625" style="7"/>
+    <col min="8" max="9" width="8.81640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="8.7265625" style="7"/>
+    <col min="12" max="12" width="8.7265625" style="7" customWidth="1"/>
+    <col min="13" max="15" width="8.81640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.90625" style="7" customWidth="1"/>
+    <col min="17" max="16384" width="8.7265625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ht="52" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="P1" s="9" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2" s="10">
+        <v>2025</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="H2" s="11">
+        <v>7465</v>
+      </c>
+      <c r="I2" s="11">
+        <v>390.74</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="L2" s="9">
+        <v>40152</v>
+      </c>
+      <c r="M2" s="12">
+        <v>275524</v>
+      </c>
+      <c r="N2" s="13">
+        <v>0.68589999999999995</v>
+      </c>
+      <c r="O2" s="6">
+        <v>30.11</v>
+      </c>
+      <c r="P2" s="12">
+        <v>228000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="H3" s="11">
+        <v>7469</v>
+      </c>
+      <c r="I3" s="11">
+        <v>481.476</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="L3" s="9">
+        <v>42688</v>
+      </c>
+      <c r="M3" s="12">
+        <v>243686</v>
+      </c>
+      <c r="N3" s="13">
+        <v>0.69410000000000005</v>
+      </c>
+      <c r="O3" s="6">
+        <v>33.57</v>
+      </c>
+      <c r="P3" s="12">
+        <v>228000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="10">
+        <v>2023</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="H4" s="11">
+        <v>7472</v>
+      </c>
+      <c r="I4" s="11">
+        <v>416.55799999999999</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="L4" s="9">
+        <v>41990</v>
+      </c>
+      <c r="M4" s="12">
+        <v>205753</v>
+      </c>
+      <c r="N4" s="13">
+        <v>0.69750000000000001</v>
+      </c>
+      <c r="O4" s="6">
+        <v>33.380000000000003</v>
+      </c>
+      <c r="P4" s="12">
+        <v>221000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5" s="10">
+        <v>2022</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="H5" s="11">
+        <v>7540</v>
+      </c>
+      <c r="I5" s="11">
+        <v>368.87299999999999</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="L5" s="9">
+        <v>47032</v>
+      </c>
+      <c r="M5" s="12">
+        <v>198298</v>
+      </c>
+      <c r="N5" s="13">
+        <v>0.6976</v>
+      </c>
+      <c r="O5" s="6">
+        <v>25.88</v>
+      </c>
+      <c r="P5" s="12">
+        <v>221000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6" s="10">
+        <v>2021</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="H6" s="11">
+        <v>7608</v>
+      </c>
+      <c r="I6" s="11">
+        <v>233.18199999999999</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="L6" s="9">
+        <v>50074</v>
+      </c>
+      <c r="M6" s="12">
+        <v>191791</v>
+      </c>
+      <c r="N6" s="13">
+        <v>0.68830000000000002</v>
+      </c>
+      <c r="O6" s="6">
+        <v>34.5</v>
+      </c>
+      <c r="P6" s="12">
+        <v>181000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7" s="10">
+        <v>2020</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="H7" s="11">
+        <v>7683</v>
+      </c>
+      <c r="I7" s="11">
+        <v>323.97500000000002</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="L7" s="9">
+        <v>59578</v>
+      </c>
+      <c r="M7" s="12">
+        <v>183007</v>
+      </c>
+      <c r="N7" s="13">
+        <v>0.6835</v>
+      </c>
+      <c r="O7" s="6">
+        <v>31.62</v>
+      </c>
+      <c r="P7" s="12">
+        <v>163000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8" s="10">
+        <v>2019</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="H8" s="11">
+        <v>7753</v>
+      </c>
+      <c r="I8" s="11">
+        <v>212.47499999999999</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="L8" s="9">
+        <v>66662</v>
+      </c>
+      <c r="M8" s="12">
+        <v>184226</v>
+      </c>
+      <c r="N8" s="13">
+        <v>0.67710000000000004</v>
+      </c>
+      <c r="O8" s="6">
+        <v>26.02</v>
+      </c>
+      <c r="P8" s="12">
+        <v>144000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9" s="10">
+        <v>2018</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="H9" s="11">
+        <v>7794</v>
+      </c>
+      <c r="I9" s="11">
+        <v>149.06899999999999</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>294</v>
+      </c>
+      <c r="L9" s="9">
+        <v>72242</v>
+      </c>
+      <c r="M9" s="12">
+        <v>176130</v>
+      </c>
+      <c r="N9" s="13">
+        <v>0.65100000000000002</v>
+      </c>
+      <c r="O9" s="6">
+        <v>21.85</v>
+      </c>
+      <c r="P9" s="12">
+        <v>131000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A10" s="10">
+        <v>2017</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="H10" s="11">
+        <v>7832</v>
+      </c>
+      <c r="I10" s="11">
+        <v>94.612300000000005</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="L10" s="9">
+        <v>76073</v>
+      </c>
+      <c r="M10" s="12">
+        <v>162601</v>
+      </c>
+      <c r="N10" s="13">
+        <v>0.64939999999999998</v>
+      </c>
+      <c r="O10" s="6">
+        <v>44.76</v>
+      </c>
+      <c r="P10" s="12">
+        <v>124000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A11" s="10">
+        <v>2016</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="H11" s="11">
+        <v>8013</v>
+      </c>
+      <c r="I11" s="11">
+        <v>78.3245</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="L11" s="9">
+        <v>40557</v>
+      </c>
+      <c r="M11" s="12">
+        <v>121471</v>
+      </c>
+      <c r="N11" s="13">
+        <v>0.64690000000000003</v>
+      </c>
+      <c r="O11" s="6">
+        <v>19.53</v>
+      </c>
+      <c r="P11" s="12">
+        <v>114000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A12" s="10">
+        <v>2015</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="H12" s="11">
+        <v>8254</v>
+      </c>
+      <c r="I12" s="11">
+        <v>55.6556</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="L12" s="9">
+        <v>27808</v>
+      </c>
+      <c r="M12" s="12">
+        <v>94389</v>
+      </c>
+      <c r="N12" s="13">
+        <v>0.64</v>
+      </c>
+      <c r="O12" s="6">
+        <v>33.130000000000003</v>
+      </c>
+      <c r="P12" s="12">
+        <v>118000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A13" s="10">
+        <v>2014</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="H13" s="11">
+        <v>8399</v>
+      </c>
+      <c r="I13" s="11">
+        <v>48.363500000000002</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>298</v>
+      </c>
+      <c r="L13" s="9">
+        <v>20645</v>
+      </c>
+      <c r="M13" s="12">
+        <v>82600</v>
+      </c>
+      <c r="N13" s="13">
+        <v>0.65739999999999998</v>
+      </c>
+      <c r="O13" s="6">
+        <v>15.89</v>
+      </c>
+      <c r="P13" s="12">
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A14" s="10">
+        <v>2013</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="H14" s="11">
+        <v>8470</v>
+      </c>
+      <c r="I14" s="11">
+        <v>39.418700000000001</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="L14" s="9">
+        <v>12601</v>
+      </c>
+      <c r="M14" s="12">
+        <v>63487</v>
+      </c>
+      <c r="N14" s="13">
+        <v>0.71240000000000003</v>
+      </c>
+      <c r="O14" s="6">
+        <v>11.49</v>
+      </c>
+      <c r="P14" s="12">
+        <v>99000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A15" s="10">
+        <v>2012</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="H15" s="11">
+        <v>8506</v>
+      </c>
+      <c r="I15" s="11">
+        <v>30.9009</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="L15" s="9">
+        <v>10713</v>
+      </c>
+      <c r="M15" s="12">
+        <v>54908</v>
+      </c>
+      <c r="N15" s="13">
+        <v>0.75349999999999995</v>
+      </c>
+      <c r="O15" s="6">
+        <v>11.7</v>
+      </c>
+      <c r="P15" s="12">
+        <v>94000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A16" s="10">
+        <v>2011</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="H16" s="11">
+        <v>8593</v>
+      </c>
+      <c r="I16" s="11">
+        <v>21.4147</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="L16" s="9">
+        <v>11921</v>
+      </c>
+      <c r="M16" s="12">
+        <v>51621</v>
+      </c>
+      <c r="N16" s="13">
+        <v>0.77200000000000002</v>
+      </c>
+      <c r="O16" s="6">
+        <v>7.33</v>
+      </c>
+      <c r="P16" s="12">
+        <v>90000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2025</v>
+      </c>
+      <c r="B2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C2" t="s">
+        <v>322</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="G2" t="s">
+        <v>385</v>
+      </c>
+      <c r="H2" s="4">
+        <v>13079</v>
+      </c>
+      <c r="I2">
+        <v>359.68</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="N2" s="5">
+        <v>0.59650000000000003</v>
+      </c>
+      <c r="O2">
+        <v>28.92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2024</v>
+      </c>
+      <c r="B3" t="s">
+        <v>307</v>
+      </c>
+      <c r="C3" t="s">
+        <v>323</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>355</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="G3" t="s">
+        <v>386</v>
+      </c>
+      <c r="H3" s="4">
+        <v>13313</v>
+      </c>
+      <c r="I3">
+        <v>312.59300000000002</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="N3" s="5">
+        <v>0.58199999999999996</v>
+      </c>
+      <c r="O3">
+        <v>23.42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2023</v>
+      </c>
+      <c r="B4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C4" t="s">
+        <v>324</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="G4" t="s">
+        <v>387</v>
+      </c>
+      <c r="H4" s="4">
+        <v>13599</v>
+      </c>
+      <c r="I4">
+        <v>188.316</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="N4" s="5">
+        <v>0.56630000000000003</v>
+      </c>
+      <c r="O4">
+        <v>23.87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2022</v>
+      </c>
+      <c r="B5" t="s">
+        <v>309</v>
+      </c>
+      <c r="C5" t="s">
+        <v>325</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="G5" t="s">
+        <v>388</v>
+      </c>
+      <c r="H5" s="4">
+        <v>14046</v>
+      </c>
+      <c r="I5">
+        <v>138.46199999999999</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="N5" s="5">
+        <v>0.55379999999999996</v>
+      </c>
+      <c r="O5">
+        <v>19.18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2021</v>
+      </c>
+      <c r="B6" t="s">
+        <v>310</v>
+      </c>
+      <c r="C6" t="s">
+        <v>326</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="G6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H6" s="4">
+        <v>14462</v>
+      </c>
+      <c r="I6">
+        <v>87.454499999999996</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="N6" s="5">
+        <v>0.56940000000000002</v>
+      </c>
+      <c r="O6">
+        <v>25.59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>2020</v>
+      </c>
+      <c r="B7" t="s">
+        <v>311</v>
+      </c>
+      <c r="C7" t="s">
+        <v>327</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="G7" t="s">
+        <v>389</v>
+      </c>
+      <c r="H7" s="4">
+        <v>14665</v>
+      </c>
+      <c r="I7">
+        <v>143.57900000000001</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="N7" s="5">
+        <v>0.53580000000000005</v>
+      </c>
+      <c r="O7">
+        <v>29.65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>2019</v>
+      </c>
+      <c r="B8" t="s">
+        <v>312</v>
+      </c>
+      <c r="C8" t="s">
+        <v>328</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="G8" t="s">
+        <v>390</v>
+      </c>
+      <c r="H8" s="4">
+        <v>14902</v>
+      </c>
+      <c r="I8">
+        <v>86.861800000000002</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="N8" s="5">
+        <v>0.55579999999999996</v>
+      </c>
+      <c r="O8">
+        <v>27.01</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>2018</v>
+      </c>
+      <c r="B9" t="s">
+        <v>313</v>
+      </c>
+      <c r="C9" t="s">
+        <v>329</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="G9" t="s">
+        <v>391</v>
+      </c>
+      <c r="H9" s="4">
+        <v>15003</v>
+      </c>
+      <c r="I9">
+        <v>66.380899999999997</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="N9" s="5">
+        <v>0.56479999999999997</v>
+      </c>
+      <c r="O9">
+        <v>23.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>2017</v>
+      </c>
+      <c r="B10" t="s">
+        <v>314</v>
+      </c>
+      <c r="C10" t="s">
+        <v>330</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="G10" t="s">
+        <v>392</v>
+      </c>
+      <c r="H10" s="4">
+        <v>15015</v>
+      </c>
+      <c r="I10">
+        <v>51.788800000000002</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="N10" s="5">
+        <v>0.58879999999999999</v>
+      </c>
+      <c r="O10">
+        <v>58.01</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>2016</v>
+      </c>
+      <c r="B11" t="s">
+        <v>315</v>
+      </c>
+      <c r="C11" t="s">
+        <v>331</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="G11" t="s">
+        <v>393</v>
+      </c>
+      <c r="H11" s="4">
+        <v>14951</v>
+      </c>
+      <c r="I11">
+        <v>52.207099999999997</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="N11" s="5">
+        <v>0.61080000000000001</v>
+      </c>
+      <c r="O11">
+        <v>28.2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>2015</v>
+      </c>
+      <c r="B12" t="s">
+        <v>316</v>
+      </c>
+      <c r="C12" t="s">
+        <v>332</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="G12" t="s">
+        <v>394</v>
+      </c>
+      <c r="H12" s="4">
+        <v>14894</v>
+      </c>
+      <c r="I12">
+        <v>39.2742</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="N12" s="5">
+        <v>0.62439999999999996</v>
+      </c>
+      <c r="O12">
+        <v>33.76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>2014</v>
+      </c>
+      <c r="B13" t="s">
+        <v>317</v>
+      </c>
+      <c r="C13" t="s">
+        <v>333</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="G13" t="s">
+        <v>395</v>
+      </c>
+      <c r="H13" s="4">
+        <v>14840</v>
+      </c>
+      <c r="I13">
+        <v>38.558599999999998</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="N13" s="5">
+        <v>0.61070000000000002</v>
+      </c>
+      <c r="O13">
+        <v>25.57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>2013</v>
+      </c>
+      <c r="B14" t="s">
+        <v>318</v>
+      </c>
+      <c r="C14" t="s">
+        <v>334</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="G14" t="s">
+        <v>396</v>
+      </c>
+      <c r="H14" s="4">
+        <v>14739</v>
+      </c>
+      <c r="I14">
+        <v>26.299800000000001</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="N14" s="5">
+        <v>0.60389999999999999</v>
+      </c>
+      <c r="O14">
+        <v>29.59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>2012</v>
+      </c>
+      <c r="B15" t="s">
+        <v>319</v>
+      </c>
+      <c r="C15" t="s">
+        <v>335</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="G15" t="s">
+        <v>397</v>
+      </c>
+      <c r="H15" s="4">
+        <v>13292</v>
+      </c>
+      <c r="I15">
+        <v>27.799299999999999</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="N15" s="5">
+        <v>0.62690000000000001</v>
+      </c>
+      <c r="O15">
+        <v>21.71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>2011</v>
+      </c>
+      <c r="B16" t="s">
+        <v>320</v>
+      </c>
+      <c r="C16" t="s">
+        <v>336</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="G16" t="s">
+        <v>398</v>
+      </c>
+      <c r="H16" s="4">
+        <v>13089</v>
+      </c>
+      <c r="I16">
+        <v>17.546600000000002</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="N16" s="5">
+        <v>0.65210000000000001</v>
+      </c>
+      <c r="O16">
+        <v>21.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>